<commit_message>
v21: mixed mounting (M10/M11/M12) - notice that per-station valve size and manifold options are not supported (all stations show the main series)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/out_filled.xlsx
+++ b/tests/out_filled.xlsx
@@ -9909,7 +9909,11 @@
       <c r="AS33" s="231"/>
       <c r="AT33" s="230"/>
       <c r="AU33" s="231"/>
-      <c r="AV33" s="230"/>
+      <c r="AV33" s="230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">○</t>
+        </is>
+      </c>
       <c r="AW33" s="231"/>
       <c r="AX33" s="230"/>
       <c r="AY33" s="231"/>
@@ -10101,11 +10105,7 @@
       <c r="AS35" s="124"/>
       <c r="AT35" s="123"/>
       <c r="AU35" s="124"/>
-      <c r="AV35" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">○</t>
-        </is>
-      </c>
+      <c r="AV35" s="123"/>
       <c r="AW35" s="124"/>
       <c r="AX35" s="123"/>
       <c r="AY35" s="124"/>
@@ -10197,7 +10197,11 @@
       <c r="AM36" s="277"/>
       <c r="AN36" s="250"/>
       <c r="AO36" s="251"/>
-      <c r="AP36" s="250"/>
+      <c r="AP36" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="AQ36" s="251"/>
       <c r="AR36" s="250"/>
       <c r="AS36" s="251"/>
@@ -10295,7 +10299,11 @@
       <c r="AM37" s="277"/>
       <c r="AN37" s="248"/>
       <c r="AO37" s="249"/>
-      <c r="AP37" s="248"/>
+      <c r="AP37" s="248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C6</t>
+        </is>
+      </c>
       <c r="AQ37" s="249"/>
       <c r="AR37" s="248"/>
       <c r="AS37" s="249"/>
@@ -10391,11 +10399,7 @@
       <c r="AM38" s="277"/>
       <c r="AN38" s="123"/>
       <c r="AO38" s="124"/>
-      <c r="AP38" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">○</t>
-        </is>
-      </c>
+      <c r="AP38" s="123"/>
       <c r="AQ38" s="124"/>
       <c r="AR38" s="123"/>
       <c r="AS38" s="124"/>

</xml_diff>